<commit_message>
Update semantic seg 2.5 benchmark results
</commit_message>
<xml_diff>
--- a/tests/perf_v2/perf_history/v2.5/semantic_segmentation/SEMANTIC_SEGMENTATION-high-level-summary.xlsx
+++ b/tests/perf_v2/perf_history/v2.5/semantic_segmentation/SEMANTIC_SEGMENTATION-high-level-summary.xlsx
@@ -496,102 +496,102 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>export:test/Dice_mean</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>export:test/Dice_std</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>export:test/e2e_time_mean</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>export:test/e2e_time_std</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>export:test/latency_mean</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>export:test/latency_std</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>torch:test/Dice_mean</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>torch:test/Dice_std</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>torch:test/iter_time_mean</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>torch:test/iter_time_std</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>torch:test/e2e_time_mean</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>torch:test/e2e_time_std</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>torch:test/latency_mean</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>torch:test/latency_std</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>optimize:test/Dice_mean</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>optimize:test/Dice_std</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>optimize:test/e2e_time_mean</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>optimize:test/e2e_time_std</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>optimize:test/latency_mean</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>optimize:test/latency_std</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>export:test/Dice_mean</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>export:test/Dice_std</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>export:test/e2e_time_mean</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>export:test/e2e_time_std</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>export:test/latency_mean</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>export:test/latency_std</t>
         </is>
       </c>
       <c r="AH1" s="1" t="inlineStr">
@@ -613,7 +613,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2.5.0dev</t>
+          <t>2.5.0</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -627,100 +627,100 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>45.5143</v>
+        <v>48.3714</v>
       </c>
       <c r="E2" t="n">
-        <v>42.0381</v>
+        <v>38.4555</v>
       </c>
       <c r="F2" t="n">
-        <v>60.0825</v>
+        <v>85.0181</v>
       </c>
       <c r="G2" t="n">
-        <v>50.284</v>
+        <v>91.5121</v>
       </c>
       <c r="H2" t="n">
-        <v>1.352</v>
+        <v>1.4234</v>
       </c>
       <c r="I2" t="n">
-        <v>0.7868000000000001</v>
+        <v>0.8498</v>
       </c>
       <c r="J2" t="n">
-        <v>0.0442</v>
+        <v>0.0439</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0113</v>
+        <v>0.0116</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7039</v>
+        <v>0.7062</v>
       </c>
       <c r="M2" t="n">
-        <v>0.1251</v>
+        <v>0.1276</v>
       </c>
       <c r="N2" t="n">
-        <v>0.6965</v>
+        <v>0.6919</v>
       </c>
       <c r="O2" t="n">
-        <v>0.1207</v>
+        <v>0.1278</v>
       </c>
       <c r="P2" t="n">
-        <v>0.0389</v>
+        <v>13.3554</v>
       </c>
       <c r="Q2" t="n">
+        <v>11.158</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.3399</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.2112</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.6998</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.1231</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.0401</v>
+      </c>
+      <c r="W2" t="n">
         <v>0.007</v>
       </c>
-      <c r="R2" t="n">
-        <v>1.6565</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0.6806</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0.082</v>
-      </c>
-      <c r="U2" t="n">
-        <v>0.0736</v>
-      </c>
-      <c r="V2" t="n">
-        <v>0.6899</v>
-      </c>
-      <c r="W2" t="n">
-        <v>0.1233</v>
-      </c>
       <c r="X2" t="n">
-        <v>14.1776</v>
+        <v>1.7</v>
       </c>
       <c r="Y2" t="n">
-        <v>14.5394</v>
+        <v>0.6892</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.4174</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.3218</v>
+        <v>0.07489999999999999</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.6901</v>
+        <v>0.6918</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.1245</v>
+        <v>0.1265</v>
       </c>
       <c r="AD2" t="n">
-        <v>13.0582</v>
+        <v>11.4466</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.8286</v>
+        <v>7.8374</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.3338</v>
+        <v>0.3709</v>
       </c>
       <c r="AG2" t="n">
-        <v>0.2088</v>
+        <v>0.2528</v>
       </c>
       <c r="AH2" t="n">
-        <v>52.2057</v>
+        <v>51.4323</v>
       </c>
       <c r="AI2" t="n">
-        <v>37.5258</v>
+        <v>37.0109</v>
       </c>
       <c r="AJ2" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2.5.0dev</t>
+          <t>2.5.0</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -745,100 +745,100 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>43.4571</v>
+        <v>64.6857</v>
       </c>
       <c r="E3" t="n">
-        <v>41.2206</v>
+        <v>31.9584</v>
       </c>
       <c r="F3" t="n">
-        <v>110.5357</v>
+        <v>418.2931</v>
       </c>
       <c r="G3" t="n">
-        <v>104.8457</v>
+        <v>571.5232</v>
       </c>
       <c r="H3" t="n">
-        <v>2.576</v>
+        <v>2.6317</v>
       </c>
       <c r="I3" t="n">
-        <v>0.5375</v>
+        <v>0.599</v>
       </c>
       <c r="J3" t="n">
-        <v>0.15</v>
+        <v>0.1566</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0056</v>
+        <v>0.0037</v>
       </c>
       <c r="L3" t="n">
-        <v>0.5279</v>
+        <v>0.6075</v>
       </c>
       <c r="M3" t="n">
-        <v>0.2634</v>
+        <v>0.2086</v>
       </c>
       <c r="N3" t="n">
-        <v>0.5193</v>
+        <v>0.5893</v>
       </c>
       <c r="O3" t="n">
-        <v>0.2505</v>
+        <v>0.1976</v>
       </c>
       <c r="P3" t="n">
-        <v>0.06560000000000001</v>
+        <v>11.3228</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.0078</v>
+        <v>7.6354</v>
       </c>
       <c r="R3" t="n">
-        <v>2.3018</v>
+        <v>0.3775</v>
       </c>
       <c r="S3" t="n">
-        <v>1.1289</v>
+        <v>0.2628</v>
       </c>
       <c r="T3" t="n">
-        <v>0.1054</v>
+        <v>0.5983000000000001</v>
       </c>
       <c r="U3" t="n">
-        <v>0.094</v>
+        <v>0.1979</v>
       </c>
       <c r="V3" t="n">
-        <v>0.5096000000000001</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="W3" t="n">
-        <v>0.2485</v>
+        <v>0.0074</v>
       </c>
       <c r="X3" t="n">
-        <v>15.2939</v>
+        <v>2.4047</v>
       </c>
       <c r="Y3" t="n">
-        <v>8.806900000000001</v>
+        <v>1.127</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.5679</v>
+        <v>0.1103</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.3918</v>
+        <v>0.09719999999999999</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.5103</v>
+        <v>0.5831</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.2465</v>
+        <v>0.2012</v>
       </c>
       <c r="AD3" t="n">
-        <v>10.9603</v>
+        <v>13.6436</v>
       </c>
       <c r="AE3" t="n">
-        <v>7.3993</v>
+        <v>7.7796</v>
       </c>
       <c r="AF3" t="n">
-        <v>0.363</v>
+        <v>0.5182</v>
       </c>
       <c r="AG3" t="n">
-        <v>0.2498</v>
+        <v>0.3743</v>
       </c>
       <c r="AH3" t="n">
-        <v>120.0993</v>
+        <v>124.0257</v>
       </c>
       <c r="AI3" t="n">
-        <v>104.199</v>
+        <v>106.7832</v>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
@@ -849,7 +849,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2.5.0dev</t>
+          <t>2.5.0</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -863,100 +863,100 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>44.0857</v>
+        <v>65.62860000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>42.0353</v>
+        <v>32.7666</v>
       </c>
       <c r="F4" t="n">
-        <v>99.65819999999999</v>
+        <v>374.6066</v>
       </c>
       <c r="G4" t="n">
-        <v>95.4926</v>
+        <v>512.0916</v>
       </c>
       <c r="H4" t="n">
-        <v>1.3489</v>
+        <v>1.4169</v>
       </c>
       <c r="I4" t="n">
-        <v>0.4563</v>
+        <v>0.5247000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1249</v>
+        <v>0.131</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0062</v>
+        <v>0.0048</v>
       </c>
       <c r="L4" t="n">
-        <v>0.4816</v>
+        <v>0.5592</v>
       </c>
       <c r="M4" t="n">
-        <v>0.2437</v>
+        <v>0.2078</v>
       </c>
       <c r="N4" t="n">
-        <v>0.48</v>
+        <v>0.5434</v>
       </c>
       <c r="O4" t="n">
-        <v>0.2385</v>
+        <v>0.2004</v>
       </c>
       <c r="P4" t="n">
-        <v>0.0586</v>
+        <v>16.6039</v>
       </c>
       <c r="Q4" t="n">
+        <v>13.0425</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.5174</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.3831</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.5542</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.1989</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.0593</v>
+      </c>
+      <c r="W4" t="n">
         <v>0.0075</v>
       </c>
-      <c r="R4" t="n">
-        <v>2.0301</v>
-      </c>
-      <c r="S4" t="n">
-        <v>0.9229000000000001</v>
-      </c>
-      <c r="T4" t="n">
-        <v>0.09909999999999999</v>
-      </c>
-      <c r="U4" t="n">
-        <v>0.0917</v>
-      </c>
-      <c r="V4" t="n">
-        <v>0.4165</v>
-      </c>
-      <c r="W4" t="n">
-        <v>0.2298</v>
-      </c>
       <c r="X4" t="n">
-        <v>20.6035</v>
+        <v>2.12</v>
       </c>
       <c r="Y4" t="n">
-        <v>13.6072</v>
+        <v>0.9888</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.7292999999999999</v>
+        <v>0.101</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.4962</v>
+        <v>0.0914</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.4706</v>
+        <v>0.4554</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.2372</v>
+        <v>0.2377</v>
       </c>
       <c r="AD4" t="n">
-        <v>16.1962</v>
+        <v>20.295</v>
       </c>
       <c r="AE4" t="n">
-        <v>12.9284</v>
+        <v>13.4086</v>
       </c>
       <c r="AF4" t="n">
-        <v>0.5013</v>
+        <v>0.7443</v>
       </c>
       <c r="AG4" t="n">
-        <v>0.3757</v>
+        <v>0.5334</v>
       </c>
       <c r="AH4" t="n">
-        <v>99.8231</v>
+        <v>103.284</v>
       </c>
       <c r="AI4" t="n">
-        <v>82.35599999999999</v>
+        <v>85.9924</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
@@ -967,7 +967,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2.5.0dev</t>
+          <t>2.5.0</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -981,100 +981,100 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>43.9143</v>
+        <v>65.0286</v>
       </c>
       <c r="E5" t="n">
-        <v>40.814</v>
+        <v>32.8262</v>
       </c>
       <c r="F5" t="n">
-        <v>236.5321</v>
+        <v>836.7761</v>
       </c>
       <c r="G5" t="n">
-        <v>293.35</v>
+        <v>1195.8639</v>
       </c>
       <c r="H5" t="n">
-        <v>8.213699999999999</v>
+        <v>8.233700000000001</v>
       </c>
       <c r="I5" t="n">
-        <v>1.1403</v>
+        <v>1.1712</v>
       </c>
       <c r="J5" t="n">
-        <v>0.3147</v>
+        <v>0.3196</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0171</v>
+        <v>0.0161</v>
       </c>
       <c r="L5" t="n">
-        <v>0.499</v>
+        <v>0.5731000000000001</v>
       </c>
       <c r="M5" t="n">
-        <v>0.2718</v>
+        <v>0.2324</v>
       </c>
       <c r="N5" t="n">
-        <v>0.4921</v>
+        <v>0.5543</v>
       </c>
       <c r="O5" t="n">
-        <v>0.2633</v>
+        <v>0.2225</v>
       </c>
       <c r="P5" t="n">
-        <v>0.1076</v>
+        <v>19.3349</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.008</v>
+        <v>14.5364</v>
       </c>
       <c r="R5" t="n">
-        <v>3.4807</v>
+        <v>0.582</v>
       </c>
       <c r="S5" t="n">
-        <v>1.743</v>
+        <v>0.3889</v>
       </c>
       <c r="T5" t="n">
-        <v>0.156</v>
+        <v>0.5656</v>
       </c>
       <c r="U5" t="n">
-        <v>0.1376</v>
+        <v>0.223</v>
       </c>
       <c r="V5" t="n">
-        <v>0.3527</v>
+        <v>0.1071</v>
       </c>
       <c r="W5" t="n">
-        <v>0.2353</v>
+        <v>0.0089</v>
       </c>
       <c r="X5" t="n">
-        <v>25.1835</v>
+        <v>3.6365</v>
       </c>
       <c r="Y5" t="n">
-        <v>12.2614</v>
+        <v>1.7675</v>
       </c>
       <c r="Z5" t="n">
-        <v>1.0581</v>
+        <v>0.1647</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.8423</v>
+        <v>0.1436</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.4817</v>
+        <v>0.3507</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.2619</v>
+        <v>0.228</v>
       </c>
       <c r="AD5" t="n">
-        <v>18.9115</v>
+        <v>25.5619</v>
       </c>
       <c r="AE5" t="n">
-        <v>14.1194</v>
+        <v>12.6495</v>
       </c>
       <c r="AF5" t="n">
-        <v>0.5666</v>
+        <v>1.0918</v>
       </c>
       <c r="AG5" t="n">
-        <v>0.3732</v>
+        <v>0.8918</v>
       </c>
       <c r="AH5" t="n">
-        <v>738.497</v>
+        <v>764.5311</v>
       </c>
       <c r="AI5" t="n">
-        <v>725.6341</v>
+        <v>752.601</v>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
@@ -1085,7 +1085,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2.5.0dev</t>
+          <t>2.5.0</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1099,100 +1099,100 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>44.6</v>
+        <v>66.8571</v>
       </c>
       <c r="E6" t="n">
-        <v>43.581</v>
+        <v>36.8216</v>
       </c>
       <c r="F6" t="n">
-        <v>146.2423</v>
+        <v>505.2147</v>
       </c>
       <c r="G6" t="n">
-        <v>139.4417</v>
+        <v>805.9921000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>7.1009</v>
+        <v>7.124</v>
       </c>
       <c r="I6" t="n">
-        <v>0.9499</v>
+        <v>0.9527</v>
       </c>
       <c r="J6" t="n">
-        <v>0.1891</v>
+        <v>0.1888</v>
       </c>
       <c r="K6" t="n">
-        <v>0.018</v>
+        <v>0.0171</v>
       </c>
       <c r="L6" t="n">
-        <v>0.5379</v>
+        <v>0.6069</v>
       </c>
       <c r="M6" t="n">
-        <v>0.2599</v>
+        <v>0.2056</v>
       </c>
       <c r="N6" t="n">
-        <v>0.5286999999999999</v>
+        <v>0.5919</v>
       </c>
       <c r="O6" t="n">
-        <v>0.2511</v>
+        <v>0.1972</v>
       </c>
       <c r="P6" t="n">
-        <v>0.07679999999999999</v>
+        <v>14.7822</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.0086</v>
+        <v>11.8462</v>
       </c>
       <c r="R6" t="n">
-        <v>2.767</v>
+        <v>0.3971</v>
       </c>
       <c r="S6" t="n">
-        <v>1.2229</v>
+        <v>0.244</v>
       </c>
       <c r="T6" t="n">
-        <v>0.1299</v>
+        <v>0.5958</v>
       </c>
       <c r="U6" t="n">
-        <v>0.1126</v>
+        <v>0.1966</v>
       </c>
       <c r="V6" t="n">
-        <v>0.5046</v>
+        <v>0.0757</v>
       </c>
       <c r="W6" t="n">
-        <v>0.2441</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="X6" t="n">
-        <v>16.4071</v>
+        <v>2.8256</v>
       </c>
       <c r="Y6" t="n">
-        <v>10.2718</v>
+        <v>1.2176</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.5889</v>
+        <v>0.1349</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.4037</v>
+        <v>0.12</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.5273</v>
+        <v>0.5593</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.2509</v>
+        <v>0.2052</v>
       </c>
       <c r="AD6" t="n">
-        <v>14.5376</v>
+        <v>14.9788</v>
       </c>
       <c r="AE6" t="n">
-        <v>11.7982</v>
+        <v>8.741300000000001</v>
       </c>
       <c r="AF6" t="n">
-        <v>0.3886</v>
+        <v>0.5735</v>
       </c>
       <c r="AG6" t="n">
-        <v>0.2423</v>
+        <v>0.4291</v>
       </c>
       <c r="AH6" t="n">
-        <v>79.9665</v>
+        <v>75.30970000000001</v>
       </c>
       <c r="AI6" t="n">
-        <v>55.5462</v>
+        <v>53.0797</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
@@ -1203,7 +1203,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2.5.0dev</t>
+          <t>2.5.0</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1217,100 +1217,100 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>44</v>
+        <v>65.48569999999999</v>
       </c>
       <c r="E7" t="n">
-        <v>42.5303</v>
+        <v>35.7025</v>
       </c>
       <c r="F7" t="n">
-        <v>96.21169999999999</v>
+        <v>326.2197</v>
       </c>
       <c r="G7" t="n">
-        <v>88.18940000000001</v>
+        <v>448.2778</v>
       </c>
       <c r="H7" t="n">
-        <v>4.3931</v>
+        <v>4.4851</v>
       </c>
       <c r="I7" t="n">
-        <v>0.7814</v>
+        <v>0.8794</v>
       </c>
       <c r="J7" t="n">
-        <v>0.1162</v>
+        <v>0.117</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0106</v>
+        <v>0.0097</v>
       </c>
       <c r="L7" t="n">
-        <v>0.5231</v>
+        <v>0.5736</v>
       </c>
       <c r="M7" t="n">
-        <v>0.2449</v>
+        <v>0.2369</v>
       </c>
       <c r="N7" t="n">
-        <v>0.5178</v>
+        <v>0.5647</v>
       </c>
       <c r="O7" t="n">
-        <v>0.2377</v>
+        <v>0.23</v>
       </c>
       <c r="P7" t="n">
-        <v>0.0532</v>
+        <v>11.0887</v>
       </c>
       <c r="Q7" t="n">
+        <v>8.5595</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.3114</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0.2031</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0.5685</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0.0533</v>
+      </c>
+      <c r="W7" t="n">
         <v>0.008500000000000001</v>
       </c>
-      <c r="R7" t="n">
-        <v>2.0204</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0.9225</v>
-      </c>
-      <c r="T7" t="n">
-        <v>0.0911</v>
-      </c>
-      <c r="U7" t="n">
-        <v>0.0767</v>
-      </c>
-      <c r="V7" t="n">
-        <v>0.5073</v>
-      </c>
-      <c r="W7" t="n">
-        <v>0.238</v>
-      </c>
       <c r="X7" t="n">
-        <v>15.4715</v>
+        <v>2.0281</v>
       </c>
       <c r="Y7" t="n">
-        <v>12.9885</v>
+        <v>0.894</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.5205</v>
+        <v>0.0959</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.3877</v>
+        <v>0.08309999999999999</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.5142</v>
+        <v>0.5506</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.2375</v>
+        <v>0.2324</v>
       </c>
       <c r="AD7" t="n">
-        <v>11.0289</v>
+        <v>11.1879</v>
       </c>
       <c r="AE7" t="n">
-        <v>8.388500000000001</v>
+        <v>7.126</v>
       </c>
       <c r="AF7" t="n">
-        <v>0.309</v>
+        <v>0.3913</v>
       </c>
       <c r="AG7" t="n">
-        <v>0.1939</v>
+        <v>0.2735</v>
       </c>
       <c r="AH7" t="n">
-        <v>47.3511</v>
+        <v>47.1312</v>
       </c>
       <c r="AI7" t="n">
-        <v>34.5522</v>
+        <v>33.7076</v>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
@@ -1321,7 +1321,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2.5.0dev</t>
+          <t>2.5.0</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1335,100 +1335,100 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>43.1714</v>
+        <v>71.94289999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>41.0219</v>
+        <v>35.9803</v>
       </c>
       <c r="F8" t="n">
-        <v>86.36199999999999</v>
+        <v>362.18</v>
       </c>
       <c r="G8" t="n">
-        <v>79.1827</v>
+        <v>505.7267</v>
       </c>
       <c r="H8" t="n">
-        <v>3.1206</v>
+        <v>3.2357</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6849</v>
+        <v>0.8008</v>
       </c>
       <c r="J8" t="n">
-        <v>0.1072</v>
+        <v>0.1087</v>
       </c>
       <c r="K8" t="n">
-        <v>0.0065</v>
+        <v>0.006</v>
       </c>
       <c r="L8" t="n">
-        <v>0.4735</v>
+        <v>0.5571</v>
       </c>
       <c r="M8" t="n">
-        <v>0.2328</v>
+        <v>0.2428</v>
       </c>
       <c r="N8" t="n">
-        <v>0.4637</v>
+        <v>0.5444</v>
       </c>
       <c r="O8" t="n">
-        <v>0.2217</v>
+        <v>0.2393</v>
       </c>
       <c r="P8" t="n">
-        <v>0.0467</v>
+        <v>10.1859</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.0083</v>
+        <v>7.4165</v>
       </c>
       <c r="R8" t="n">
-        <v>1.7896</v>
+        <v>0.3124</v>
       </c>
       <c r="S8" t="n">
-        <v>0.7892</v>
+        <v>0.2181</v>
       </c>
       <c r="T8" t="n">
-        <v>0.0832</v>
+        <v>0.5513</v>
       </c>
       <c r="U8" t="n">
-        <v>0.0707</v>
+        <v>0.237</v>
       </c>
       <c r="V8" t="n">
-        <v>0.4402</v>
+        <v>0.0473</v>
       </c>
       <c r="W8" t="n">
-        <v>0.2286</v>
+        <v>0.0075</v>
       </c>
       <c r="X8" t="n">
-        <v>12.1297</v>
+        <v>1.7861</v>
       </c>
       <c r="Y8" t="n">
-        <v>9.613</v>
+        <v>0.7954</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.4316</v>
+        <v>0.0837</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.3102</v>
+        <v>0.0722</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.4583</v>
+        <v>0.5375</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.2226</v>
+        <v>0.2385</v>
       </c>
       <c r="AD8" t="n">
-        <v>9.8064</v>
+        <v>11.4316</v>
       </c>
       <c r="AE8" t="n">
-        <v>7.0969</v>
+        <v>6.947</v>
       </c>
       <c r="AF8" t="n">
-        <v>0.2986</v>
+        <v>0.4239</v>
       </c>
       <c r="AG8" t="n">
-        <v>0.2058</v>
+        <v>0.3053</v>
       </c>
       <c r="AH8" t="n">
-        <v>38.9312</v>
+        <v>41.31</v>
       </c>
       <c r="AI8" t="n">
-        <v>23.2579</v>
+        <v>26.7382</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>

</xml_diff>